<commit_message>
feat: Depression Screening quality measure — 7 statuses, color coding, import support, seed data (+14 Vitest)
Add Depression Screening as a new Screening-type quality measure with full stack support:
- 7 statuses with color coding (white/blue/yellow/green/gray/purple) and overdue timers
- Hill import column mapping + Sutter regex action pattern (Depression Screening, PHQ-9, Screen for depression)
- Date prompts, seed patients/measures, validator, test data fixtures
- 14 new Vitest tests covering dropdown config, status colors, filter integration, and import pipeline

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/test-data/test-sutter-valid.xlsx
+++ b/test-data/test-sutter-valid.xlsx
@@ -400,7 +400,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:J22"/>
+  <dimension ref="A1:J25"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -899,16 +899,16 @@
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>Harris, Pat</v>
+        <v>Hill, Nancy</v>
       </c>
       <c r="B19" t="str">
-        <v>04/10/1979</v>
+        <v>05/20/1985</v>
       </c>
       <c r="C19" t="str">
-        <v>(555) 100-0008</v>
+        <v>(555) 100-0010</v>
       </c>
       <c r="D19" t="str">
-        <v>800 Walnut Blvd</v>
+        <v>1000 Poplar Dr</v>
       </c>
       <c r="E19" t="str">
         <v>Plan A</v>
@@ -917,10 +917,10 @@
         <v>White</v>
       </c>
       <c r="G19" t="str">
-        <v/>
+        <v>Depression Screening due in 2025</v>
       </c>
       <c r="H19" t="str">
-        <v>AWV</v>
+        <v>Quality</v>
       </c>
       <c r="I19" t="str">
         <v/>
@@ -931,16 +931,16 @@
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>Harris, Pat</v>
+        <v>Hill, Nancy</v>
       </c>
       <c r="B20" t="str">
-        <v>04/10/1979</v>
+        <v>05/20/1985</v>
       </c>
       <c r="C20" t="str">
-        <v>(555) 100-0008</v>
+        <v>(555) 100-0010</v>
       </c>
       <c r="D20" t="str">
-        <v>800 Walnut Blvd</v>
+        <v>1000 Poplar Dr</v>
       </c>
       <c r="E20" t="str">
         <v>Plan A</v>
@@ -949,13 +949,13 @@
         <v>White</v>
       </c>
       <c r="G20" t="str">
-        <v>FOBT in 2025 or colonoscopy</v>
+        <v>PHQ-9 screening needed</v>
       </c>
       <c r="H20" t="str">
         <v>Quality</v>
       </c>
       <c r="I20" t="str">
-        <v>01/15/2025, 03/20/2025</v>
+        <v/>
       </c>
       <c r="J20" t="str">
         <v>N</v>
@@ -963,16 +963,16 @@
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>Irving, Kim</v>
+        <v>James, Oliver</v>
       </c>
       <c r="B21" t="str">
-        <v>08/18/1990</v>
+        <v>09/14/1972</v>
       </c>
       <c r="C21" t="str">
-        <v>(555) 100-0009</v>
+        <v>(555) 100-0011</v>
       </c>
       <c r="D21" t="str">
-        <v>900 Ash St</v>
+        <v>1100 Magnolia Ave</v>
       </c>
       <c r="E21" t="str">
         <v>Plan A</v>
@@ -981,7 +981,7 @@
         <v>White</v>
       </c>
       <c r="G21" t="str">
-        <v>Mammogram in 2025</v>
+        <v>Screen for depression in 2025</v>
       </c>
       <c r="H21" t="str">
         <v>Quality</v>
@@ -995,46 +995,142 @@
     </row>
     <row r="22">
       <c r="A22" t="str">
+        <v>Harris, Pat</v>
+      </c>
+      <c r="B22" t="str">
+        <v>04/10/1979</v>
+      </c>
+      <c r="C22" t="str">
+        <v>(555) 100-0008</v>
+      </c>
+      <c r="D22" t="str">
+        <v>800 Walnut Blvd</v>
+      </c>
+      <c r="E22" t="str">
+        <v>Plan A</v>
+      </c>
+      <c r="F22" t="str">
+        <v>White</v>
+      </c>
+      <c r="G22" t="str">
+        <v/>
+      </c>
+      <c r="H22" t="str">
+        <v>AWV</v>
+      </c>
+      <c r="I22" t="str">
+        <v/>
+      </c>
+      <c r="J22" t="str">
+        <v>N</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="str">
+        <v>Harris, Pat</v>
+      </c>
+      <c r="B23" t="str">
+        <v>04/10/1979</v>
+      </c>
+      <c r="C23" t="str">
+        <v>(555) 100-0008</v>
+      </c>
+      <c r="D23" t="str">
+        <v>800 Walnut Blvd</v>
+      </c>
+      <c r="E23" t="str">
+        <v>Plan A</v>
+      </c>
+      <c r="F23" t="str">
+        <v>White</v>
+      </c>
+      <c r="G23" t="str">
+        <v>FOBT in 2025 or colonoscopy</v>
+      </c>
+      <c r="H23" t="str">
+        <v>Quality</v>
+      </c>
+      <c r="I23" t="str">
+        <v>01/15/2025, 03/20/2025</v>
+      </c>
+      <c r="J23" t="str">
+        <v>N</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="str">
         <v>Irving, Kim</v>
       </c>
-      <c r="B22" t="str">
+      <c r="B24" t="str">
         <v>08/18/1990</v>
       </c>
-      <c r="C22" t="str">
+      <c r="C24" t="str">
         <v>(555) 100-0009</v>
       </c>
-      <c r="D22" t="str">
+      <c r="D24" t="str">
         <v>900 Ash St</v>
       </c>
-      <c r="E22" t="str">
-        <v>Plan A</v>
-      </c>
-      <c r="F22" t="str">
-        <v>White</v>
-      </c>
-      <c r="G22" t="str">
+      <c r="E24" t="str">
+        <v>Plan A</v>
+      </c>
+      <c r="F24" t="str">
+        <v>White</v>
+      </c>
+      <c r="G24" t="str">
+        <v>Mammogram in 2025</v>
+      </c>
+      <c r="H24" t="str">
+        <v>Quality</v>
+      </c>
+      <c r="I24" t="str">
+        <v/>
+      </c>
+      <c r="J24" t="str">
+        <v>N</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="str">
+        <v>Irving, Kim</v>
+      </c>
+      <c r="B25" t="str">
+        <v>08/18/1990</v>
+      </c>
+      <c r="C25" t="str">
+        <v>(555) 100-0009</v>
+      </c>
+      <c r="D25" t="str">
+        <v>900 Ash St</v>
+      </c>
+      <c r="E25" t="str">
+        <v>Plan A</v>
+      </c>
+      <c r="F25" t="str">
+        <v>White</v>
+      </c>
+      <c r="G25" t="str">
         <v>Vaccine: Tdap shot due</v>
       </c>
-      <c r="H22" t="str">
-        <v>Quality</v>
-      </c>
-      <c r="I22" t="str">
-        <v/>
-      </c>
-      <c r="J22" t="str">
+      <c r="H25" t="str">
+        <v>Quality</v>
+      </c>
+      <c r="I25" t="str">
+        <v/>
+      </c>
+      <c r="J25" t="str">
         <v>N</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:J22"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:J25"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:J12"/>
+  <dimension ref="A1:J13"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1339,9 +1435,41 @@
         <v>N</v>
       </c>
     </row>
+    <row r="13">
+      <c r="A13" t="str">
+        <v>Nelson, Grace</v>
+      </c>
+      <c r="B13" t="str">
+        <v>07/15/1978</v>
+      </c>
+      <c r="C13" t="str">
+        <v>(555) 200-0005</v>
+      </c>
+      <c r="D13" t="str">
+        <v>1400 Aspen Way</v>
+      </c>
+      <c r="E13" t="str">
+        <v>Plan A</v>
+      </c>
+      <c r="F13" t="str">
+        <v>White</v>
+      </c>
+      <c r="G13" t="str">
+        <v>Depression screening in 2025</v>
+      </c>
+      <c r="H13" t="str">
+        <v>Quality</v>
+      </c>
+      <c r="I13" t="str">
+        <v/>
+      </c>
+      <c r="J13" t="str">
+        <v>N</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:J12"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:J13"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>